<commit_message>
feat: add initial dish seed data and images
</commit_message>
<xml_diff>
--- a/docs/THAI_TABE_TOKYO_初期登録データ.xlsx
+++ b/docs/THAI_TABE_TOKYO_初期登録データ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yukari\Desktop\thai-tabe-tokyo\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56980ABE-CE05-42B2-A47C-94C6EC4830F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEAC8A72-0AAC-44AE-BB33-7CE0D3AEDB62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8010" yWindow="585" windowWidth="20790" windowHeight="14250" xr2:uid="{5D5CEF65-7EB7-4E03-A33E-EA327AF4B51E}"/>
+    <workbookView xWindow="8010" yWindow="585" windowWidth="20790" windowHeight="14250" activeTab="1" xr2:uid="{5D5CEF65-7EB7-4E03-A33E-EA327AF4B51E}"/>
   </bookViews>
   <sheets>
     <sheet name="エリア" sheetId="5" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="68">
   <si>
     <t>area_id</t>
   </si>
@@ -239,13 +239,29 @@
   </si>
   <si>
     <t>alt_text</t>
+  </si>
+  <si>
+    <t>https://lziiorwcgjeeuyafrjyq.supabase.co/storage/v1/object/public/thai-tabe-images/dishes/gapao.jpg</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>https://lziiorwcgjeeuyafrjyq.supabase.co/storage/v1/object/public/thai-tabe-images/dishes/khao-man-gai.jpg</t>
+  </si>
+  <si>
+    <t>https://lziiorwcgjeeuyafrjyq.supabase.co/storage/v1/object/public/thai-tabe-images/dishes/pad-thai.jpg</t>
+  </si>
+  <si>
+    <t>https://lziiorwcgjeeuyafrjyq.supabase.co/storage/v1/object/public/thai-tabe-images/dishes/thai-curry.jpg</t>
+  </si>
+  <si>
+    <t>https://lziiorwcgjeeuyafrjyq.supabase.co/storage/v1/object/public/thai-tabe-images/dishes/tom-yum-goong.jpg</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -270,6 +286,12 @@
       <charset val="128"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="6"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -293,12 +315,15 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -784,7 +809,7 @@
     <col min="1" max="1" width="10.125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.75" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="29.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.75" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37" customWidth="1"/>
     <col min="5" max="5" width="16.375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.75" bestFit="1" customWidth="1"/>
   </cols>
@@ -809,13 +834,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" ht="73.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2">
+        <v>1</v>
+      </c>
       <c r="B2" t="s">
         <v>16</v>
       </c>
       <c r="C2" t="s">
         <v>17</v>
       </c>
+      <c r="D2" s="2" t="s">
+        <v>63</v>
+      </c>
       <c r="E2">
         <v>1</v>
       </c>
@@ -823,13 +854,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" ht="66.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3">
+        <v>2</v>
+      </c>
       <c r="B3" t="s">
         <v>18</v>
       </c>
       <c r="C3" t="s">
         <v>19</v>
       </c>
+      <c r="D3" s="2" t="s">
+        <v>64</v>
+      </c>
       <c r="E3">
         <v>2</v>
       </c>
@@ -837,13 +874,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" ht="72.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4">
+        <v>3</v>
+      </c>
       <c r="B4" t="s">
         <v>20</v>
       </c>
       <c r="C4" t="s">
         <v>21</v>
       </c>
+      <c r="D4" s="2" t="s">
+        <v>65</v>
+      </c>
       <c r="E4">
         <v>3</v>
       </c>
@@ -851,13 +894,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" ht="82.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5">
+        <v>4</v>
+      </c>
       <c r="B5" t="s">
         <v>22</v>
       </c>
       <c r="C5" t="s">
         <v>23</v>
       </c>
+      <c r="D5" s="2" t="s">
+        <v>66</v>
+      </c>
       <c r="E5">
         <v>4</v>
       </c>
@@ -865,13 +914,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" ht="83.25" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6">
+        <v>5</v>
+      </c>
       <c r="B6" t="s">
         <v>24</v>
       </c>
       <c r="C6" t="s">
         <v>25</v>
       </c>
+      <c r="D6" s="2" t="s">
+        <v>67</v>
+      </c>
       <c r="E6">
         <v>5</v>
       </c>
@@ -880,6 +935,9 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A7">
+        <v>6</v>
+      </c>
       <c r="B7" t="s">
         <v>26</v>
       </c>

</xml_diff>

<commit_message>
feat: add store dish and photo seed data
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/THAI_TABE_TOKYO_初期登録データ.xlsx
+++ b/docs/THAI_TABE_TOKYO_初期登録データ.xlsx
@@ -5651,7 +5651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D228"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18.75"/>
   <cols>
     <col width="11.125" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -5680,6 +5680,3184 @@
         <is>
           <t>is_available</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C13" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D13" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C17" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C18" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D18" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C22" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D22" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C23" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D23" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C24" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D24" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C26" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C28" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D28" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C29" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D29" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C30" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D30" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C32" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D32" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C33" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D33" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C34" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D34" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C35" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D35" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C36" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D36" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C38" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C39" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C40" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D40" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C41" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D41" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C42" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D42" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C44" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D44" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C45" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D45" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C46" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D46" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C47" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D47" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C48" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D48" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C50" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D50" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C51" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D51" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B52" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C52" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D52" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B53" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C53" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D53" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B54" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C54" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D54" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B55" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C55" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B56" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C56" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B57" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C57" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D57" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B58" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C58" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D58" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B59" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C59" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D59" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B60" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C60" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D60" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B61" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C61" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B62" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C62" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D62" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B63" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C63" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D63" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B64" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C64" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D64" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B65" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C65" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D65" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B66" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C66" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D66" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B67" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B68" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C68" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D68" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B69" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C69" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D69" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B70" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C70" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D70" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B71" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C71" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D71" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B72" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C72" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D72" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B73" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C73" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D73" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B74" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C74" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D74" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B75" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C75" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D75" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B76" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C76" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D76" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B77" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C77" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D77" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B78" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C78" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D78" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B79" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C79" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D79" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B80" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C80" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D80" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B81" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C81" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D81" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B82" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C82" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D82" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B83" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C83" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D83" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B84" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C84" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D84" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B85" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C85" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D85" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B86" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C86" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D86" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B87" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C87" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D87" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B88" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C88" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D88" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B89" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C89" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D89" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B90" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C90" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D90" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B91" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C91" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D91" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B92" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C92" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D92" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B93" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C93" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D93" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B94" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C94" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D94" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B95" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C95" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D95" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B96" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C96" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D96" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B97" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C97" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D97" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B98" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C98" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D98" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B99" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C99" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D99" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B100" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C100" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D100" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B101" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C101" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D101" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B102" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C102" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D102" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B103" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C103" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D103" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B104" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C104" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D104" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B105" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C105" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D105" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B106" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C106" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D106" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B107" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C107" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D107" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B108" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C108" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D108" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B109" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C109" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D109" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B110" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C110" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D110" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B111" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C111" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D111" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B112" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C112" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D112" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B113" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C113" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D113" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B114" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C114" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D114" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B115" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C115" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D115" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B116" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C116" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D116" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B117" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C117" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D117" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B118" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C118" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D118" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B119" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C119" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D119" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B120" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C120" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D120" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B121" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C121" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D121" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B122" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C122" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D122" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B123" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C123" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D123" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B124" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C124" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D124" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B125" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C125" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D125" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B126" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C126" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D126" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B127" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C127" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D127" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B128" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C128" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D128" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B129" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C129" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D129" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B130" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C130" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D130" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B131" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C131" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D131" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B132" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C132" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D132" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B133" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C133" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D133" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B134" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C134" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D134" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B135" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C135" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D135" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B136" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C136" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D136" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B137" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C137" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D137" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B138" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C138" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D138" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B139" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C139" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D139" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B140" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C140" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D140" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B141" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C141" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D141" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B142" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C142" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D142" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B143" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C143" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D143" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B144" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C144" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D144" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B145" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C145" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D145" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B146" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C146" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D146" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B147" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C147" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D147" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B148" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C148" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D148" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B149" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C149" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D149" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B150" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C150" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D150" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B151" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C151" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D151" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B152" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C152" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D152" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B153" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C153" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D153" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B154" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C154" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D154" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B155" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C155" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D155" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B156" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C156" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D156" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B157" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C157" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D157" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B158" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C158" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D158" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B159" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C159" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D159" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B160" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C160" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D160" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B161" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C161" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D161" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B162" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C162" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D162" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B163" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C163" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D163" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B164" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C164" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D164" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B165" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C165" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D165" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B166" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C166" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D166" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B167" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C167" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D167" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B168" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C168" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D168" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B169" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C169" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D169" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B170" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C170" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D170" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B171" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C171" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D171" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B172" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C172" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D172" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B173" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C173" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D173" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B174" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C174" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D174" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B175" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C175" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D175" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B176" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C176" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D176" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B177" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C177" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D177" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B178" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C178" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D178" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B179" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C179" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D179" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B180" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C180" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D180" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B181" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C181" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D181" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B182" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C182" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D182" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B183" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C183" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D183" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B184" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C184" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D184" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B185" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C185" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D185" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B186" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C186" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D186" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B187" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C187" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D187" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B188" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C188" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D188" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B189" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C189" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D189" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B190" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C190" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D190" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B191" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C191" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D191" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B192" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C192" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D192" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B193" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C193" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D193" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B194" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C194" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D194" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B195" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C195" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D195" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B196" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C196" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D196" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B197" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C197" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D197" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B198" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C198" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D198" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B199" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C199" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D199" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B200" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C200" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D200" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B201" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C201" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D201" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B202" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C202" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D202" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B203" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C203" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D203" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B204" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C204" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D204" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B205" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C205" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D205" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B206" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C206" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D206" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B207" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C207" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D207" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B208" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C208" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D208" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B209" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C209" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D209" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B210" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C210" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D210" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B211" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C211" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D211" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B212" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C212" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D212" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B213" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C213" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D213" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B214" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C214" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D214" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B215" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C215" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D215" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B216" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C216" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D216" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B217" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C217" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D217" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B218" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C218" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D218" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B219" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C219" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D219" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B220" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C220" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D220" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B221" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C221" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D221" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B222" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C222" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D222" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B223" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C223" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D223" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B224" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C224" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D224" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B225" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C225" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D225" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B226" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C226" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D226" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B227" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C227" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D227" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B228" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C228" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D228" s="0" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -5694,7 +8872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18.75"/>
   <cols>
     <col width="11.625" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -5743,6 +8921,78 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>外観</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://lziiorwcgjeeuyafrjyq.supabase.co/storage/v1/object/public/thai-tabe-images/stores/store-001-exterior-01.png</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>タイ料理店の外観イメージ（AI生成）</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>店内</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://lziiorwcgjeeuyafrjyq.supabase.co/storage/v1/object/public/thai-tabe-images/stores/store-001-interior-01.png</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>タイ料理店の店内イメージ（AI生成）</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>料理</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://lziiorwcgjeeuyafrjyq.supabase.co/storage/v1/object/public/thai-tabe-images/stores/store-001-gapao-01.png</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ガパオの料理イメージ（AI生成）</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>